<commit_message>
Fix preview indexing, case references, and PDF downloads
</commit_message>
<xml_diff>
--- a/data/import/vegan-leather/vegan-leather.xlsx
+++ b/data/import/vegan-leather/vegan-leather.xlsx
@@ -5196,19 +5196,21 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warp ≥ 30% / Weft ≥ 40%</t>
+          <t>Warp 80% / Weft 150%</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">縦 ≥ 30% / 横 ≥ 40%</t>
+          <t>縦 80% / 横 150%</t>
         </is>
       </c>
       <c r="I6" s="3" t="str">
         <v>断裂伸长率</v>
       </c>
-      <c r="J6" s="3" t="str">
-        <v>经向 ≥ 30% / 纬向 ≥ 40%</v>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>经向 80% / 纬向 150%</t>
+        </is>
       </c>
     </row>
     <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="7" ht="24" customHeight="1">

</xml_diff>